<commit_message>
Corrige porte de empresas: MEI/ME-EPP/Grande-Médio real (não MEI vs Demais)
Descobri que dá pra derivar o porte real sem precisar do arquivo EMPRESAS
da Receita (que não tinha sido baixado): o campo "Opção pelo Simples
Nacional" do arquivo SIMPLES já serve de proxy padrão, já que só empresa
de faturamento baixo pode optar pelo Simples.

- MEI: optante pelo MEI
- ME/EPP: optante pelo Simples Nacional, mas não MEI
- Grande/Médio: não optante pelo Simples Nacional

Reprocessei o staging do CNPJ (matriz, 17GB) com esse campo e refiz todas
as planilhas afetadas: Empresas_Ativas_completo, QL_por_Grupo_CNAE,
Empresas_por_Secao/Divisao/Grupo, QL_Grupo_Empresas_por_Porte (agora com
abas MEI/MEEPP/GrandeMedio em vez de MEI/Demais), Estoque_Empresas,
Empresas_e_QL master workbook. Testado no painel Streamlit — pizza de
porte mostra os 3 valores reais.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Estoque_Empresas_Ananindeua_Capanema.xlsx
+++ b/Estoque_Empresas_Ananindeua_Capanema.xlsx
@@ -561,26 +561,26 @@
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>1428.6%</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -596,26 +596,26 @@
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I5" s="9" t="inlineStr">
         <is>
-          <t>200.0%</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -631,26 +631,26 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>117</v>
+        <v>99</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>156</v>
+        <v>133</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>286</v>
+        <v>259</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>661</v>
+        <v>627</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>1383</v>
+        <v>1339</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>3194</v>
+        <v>3128</v>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>2629.9%</t>
+          <t>3059.6%</t>
         </is>
       </c>
     </row>
@@ -666,26 +666,26 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>87.5%</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -701,26 +701,26 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>2366.7%</t>
+          <t>2660.0%</t>
         </is>
       </c>
     </row>
@@ -736,26 +736,26 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>246</v>
+        <v>222</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>490</v>
+        <v>448</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>1081</v>
+        <v>1026</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>2594</v>
+        <v>2496</v>
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>2468.3%</t>
+          <t>2583.9%</t>
         </is>
       </c>
     </row>
@@ -771,26 +771,26 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>420</v>
+        <v>367</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>674</v>
+        <v>582</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>1250</v>
+        <v>1105</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>2719</v>
+        <v>2491</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>5947</v>
+        <v>5522</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>12815</v>
+        <v>12046</v>
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>2951.2%</t>
+          <t>3182.3%</t>
         </is>
       </c>
     </row>
@@ -806,26 +806,26 @@
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>95</v>
+        <v>62</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>173</v>
+        <v>122</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>372</v>
+        <v>309</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>955</v>
+        <v>868</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>4350</v>
+        <v>4209</v>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>7667.9%</t>
+          <t>10165.9%</t>
         </is>
       </c>
     </row>
@@ -844,23 +844,23 @@
         <v>16</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>1032</v>
+        <v>1006</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>3270</v>
+        <v>3213</v>
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>20337.5%</t>
+          <t>19981.2%</t>
         </is>
       </c>
     </row>
@@ -882,20 +882,20 @@
         <v>17</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>590</v>
+        <v>574</v>
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>5800.0%</t>
+          <t>5640.0%</t>
         </is>
       </c>
     </row>
@@ -911,26 +911,26 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="D14" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="D14" s="7" t="n">
-        <v>26</v>
-      </c>
       <c r="E14" s="7" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>204</v>
+        <v>175</v>
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>1033.3%</t>
+          <t>1490.9%</t>
         </is>
       </c>
     </row>
@@ -946,26 +946,26 @@
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>1180.0%</t>
+          <t>1250.0%</t>
         </is>
       </c>
     </row>
@@ -981,26 +981,26 @@
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>784</v>
+        <v>779</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>2328</v>
+        <v>2310</v>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>8214.3%</t>
+          <t>8455.6%</t>
         </is>
       </c>
     </row>
@@ -1016,26 +1016,26 @@
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>430</v>
+        <v>414</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>902</v>
+        <v>866</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>2191</v>
+        <v>2120</v>
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>3122.1%</t>
+          <t>3161.5%</t>
         </is>
       </c>
     </row>
@@ -1051,26 +1051,26 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D18" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="D18" s="7" t="n">
-        <v>14</v>
-      </c>
       <c r="E18" s="7" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>487.5%</t>
+          <t>720.0%</t>
         </is>
       </c>
     </row>
@@ -1086,26 +1086,26 @@
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>233</v>
+        <v>213</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>482</v>
+        <v>449</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>1408</v>
+        <v>1356</v>
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>2773.5%</t>
+          <t>3290.0%</t>
         </is>
       </c>
     </row>
@@ -1121,26 +1121,26 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>165</v>
+        <v>127</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>292</v>
+        <v>237</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>767</v>
+        <v>683</v>
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>2544.8%</t>
+          <t>3152.4%</t>
         </is>
       </c>
     </row>
@@ -1156,26 +1156,26 @@
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>418</v>
+        <v>408</v>
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>1572.0%</t>
+          <t>1600.0%</t>
         </is>
       </c>
     </row>
@@ -1191,26 +1191,26 @@
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>295</v>
+        <v>224</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>372</v>
+        <v>288</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>505</v>
+        <v>410</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>861</v>
+        <v>739</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>1683</v>
+        <v>1539</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>3520</v>
+        <v>3344</v>
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>1093.2%</t>
+          <t>1392.9%</t>
         </is>
       </c>
     </row>
@@ -1292,26 +1292,26 @@
       </c>
       <c r="B25" s="9" t="n"/>
       <c r="C25" s="9" t="n">
-        <v>1278</v>
+        <v>1062</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>1884</v>
+        <v>1575</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>3284</v>
+        <v>2843</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>6888</v>
+        <v>6258</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>15277</v>
+        <v>14275</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>38319</v>
+        <v>36590</v>
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>2898.4%</t>
+          <t>3345.4%</t>
         </is>
       </c>
     </row>
@@ -1424,26 +1424,26 @@
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>766.7%</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1459,26 +1459,26 @@
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="I5" s="9" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1494,26 +1494,26 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>353</v>
+        <v>344</v>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>3822.2%</t>
+          <t>4814.3%</t>
         </is>
       </c>
     </row>
@@ -1529,26 +1529,26 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1564,26 +1564,26 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F8" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G8" s="7" t="n">
-        <v>5</v>
-      </c>
       <c r="H8" s="7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>300.0%</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1599,26 +1599,26 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>3816.7%</t>
+          <t>5675.0%</t>
         </is>
       </c>
     </row>
@@ -1634,26 +1634,26 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>249</v>
+        <v>230</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>637</v>
+        <v>599</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>1267</v>
+        <v>1204</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>2446</v>
+        <v>2315</v>
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>3297.2%</t>
+          <t>3517.2%</t>
         </is>
       </c>
     </row>
@@ -1669,26 +1669,26 @@
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>315</v>
+        <v>290</v>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>5150.0%</t>
+          <t>7150.0%</t>
         </is>
       </c>
     </row>
@@ -1716,14 +1716,14 @@
         <v>69</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>368</v>
+        <v>360</v>
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>36700.0%</t>
+          <t>35900.0%</t>
         </is>
       </c>
     </row>
@@ -1745,20 +1745,20 @@
         <v>2</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>2850.0%</t>
+          <t>2400.0%</t>
         </is>
       </c>
     </row>
@@ -1774,26 +1774,26 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="E14" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="G14" s="7" t="n">
-        <v>13</v>
-      </c>
       <c r="H14" s="7" t="n">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>440.0%</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1824,11 +1824,11 @@
         <v>14</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>900.0%</t>
+          <t>850.0%</t>
         </is>
       </c>
     </row>
@@ -1853,17 +1853,17 @@
         <v>27</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>3070.0%</t>
+          <t>3000.0%</t>
         </is>
       </c>
     </row>
@@ -1882,23 +1882,23 @@
         <v>4</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>5825.0%</t>
+          <t>5550.0%</t>
         </is>
       </c>
     </row>
@@ -1914,26 +1914,26 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D18" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="D18" s="7" t="n">
-        <v>11</v>
-      </c>
       <c r="E18" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="G18" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="G18" s="7" t="n">
-        <v>14</v>
-      </c>
       <c r="H18" s="7" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>62.5%</t>
         </is>
       </c>
     </row>
@@ -1949,26 +1949,26 @@
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>1750.0%</t>
+          <t>2150.0%</t>
         </is>
       </c>
     </row>
@@ -1990,20 +1990,20 @@
         <v>9</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>125</v>
+        <v>108</v>
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>3025.0%</t>
+          <t>2600.0%</t>
         </is>
       </c>
     </row>
@@ -2028,17 +2028,17 @@
         <v>5</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>2000.0%</t>
+          <t>1933.3%</t>
         </is>
       </c>
     </row>
@@ -2054,26 +2054,26 @@
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>334</v>
+        <v>325</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>513</v>
+        <v>501</v>
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>654.4%</t>
+          <t>695.2%</t>
         </is>
       </c>
     </row>
@@ -2155,26 +2155,26 @@
       </c>
       <c r="B25" s="9" t="n"/>
       <c r="C25" s="9" t="n">
-        <v>219</v>
+        <v>182</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>334</v>
+        <v>284</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>612</v>
+        <v>546</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>1402</v>
+        <v>1303</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>2695</v>
+        <v>2538</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>5306</v>
+        <v>5008</v>
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>2322.8%</t>
+          <t>2651.6%</t>
         </is>
       </c>
     </row>
@@ -2287,26 +2287,26 @@
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>473</v>
+        <v>0</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>634</v>
+        <v>0</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>906</v>
+        <v>0</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1323</v>
+        <v>0</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>2084</v>
+        <v>0</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>5263</v>
+        <v>0</v>
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>1012.7%</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2322,26 +2322,26 @@
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>144</v>
+        <v>0</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>235</v>
+        <v>0</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>344</v>
+        <v>0</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>518</v>
+        <v>0</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>842</v>
+        <v>0</v>
       </c>
       <c r="I5" s="9" t="inlineStr">
         <is>
-          <t>750.5%</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2357,26 +2357,26 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>1264</v>
+        <v>1062</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>1835</v>
+        <v>1571</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>3228</v>
+        <v>2875</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>7019</v>
+        <v>6544</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>14483</v>
+        <v>13846</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>32604</v>
+        <v>31574</v>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>2479.4%</t>
+          <t>2873.1%</t>
         </is>
       </c>
     </row>
@@ -2392,26 +2392,26 @@
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>222</v>
+        <v>3</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>274</v>
+        <v>6</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>288</v>
+        <v>14</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>308</v>
+        <v>22</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>361</v>
+        <v>47</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>478</v>
+        <v>93</v>
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>115.3%</t>
+          <t>3000.0%</t>
         </is>
       </c>
     </row>
@@ -2427,26 +2427,26 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>107</v>
+        <v>34</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>137</v>
+        <v>61</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>190</v>
+        <v>106</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>320</v>
+        <v>226</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>565</v>
+        <v>460</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>1270</v>
+        <v>1119</v>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>1086.9%</t>
+          <t>3191.2%</t>
         </is>
       </c>
     </row>
@@ -2462,26 +2462,26 @@
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>904</v>
+        <v>808</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>1421</v>
+        <v>1295</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>2486</v>
+        <v>2282</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>5381</v>
+        <v>4993</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>11241</v>
+        <v>10674</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>26836</v>
+        <v>25822</v>
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>2868.6%</t>
+          <t>3095.8%</t>
         </is>
       </c>
     </row>
@@ -2497,26 +2497,26 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>6795</v>
+        <v>6030</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>10932</v>
+        <v>9734</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>19322</v>
+        <v>17446</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>40328</v>
+        <v>37187</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>82502</v>
+        <v>77046</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>178329</v>
+        <v>167566</v>
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>2524.4%</t>
+          <t>2678.9%</t>
         </is>
       </c>
     </row>
@@ -2532,26 +2532,26 @@
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>786</v>
+        <v>468</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>1191</v>
+        <v>733</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>1931</v>
+        <v>1321</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>3869</v>
+        <v>3014</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>8921</v>
+        <v>7698</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>30574</v>
+        <v>28433</v>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>3789.8%</t>
+          <t>5975.4%</t>
         </is>
       </c>
     </row>
@@ -2567,26 +2567,26 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>502</v>
+        <v>471</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>779</v>
+        <v>734</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>1538</v>
+        <v>1449</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>4474</v>
+        <v>4313</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>12195</v>
+        <v>11866</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>35276</v>
+        <v>34422</v>
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>6927.1%</t>
+          <t>7208.3%</t>
         </is>
       </c>
     </row>
@@ -2602,26 +2602,26 @@
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>262</v>
+        <v>245</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>398</v>
+        <v>373</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>686</v>
+        <v>636</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>1327</v>
+        <v>1207</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>2955</v>
+        <v>2673</v>
       </c>
       <c r="H13" s="9" t="n">
-        <v>7580</v>
+        <v>6985</v>
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>2793.1%</t>
+          <t>2751.0%</t>
         </is>
       </c>
     </row>
@@ -2637,26 +2637,26 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>449</v>
+        <v>196</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>607</v>
+        <v>296</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>804</v>
+        <v>407</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>1227</v>
+        <v>625</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>1745</v>
+        <v>1000</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>3257</v>
+        <v>2264</v>
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>625.4%</t>
+          <t>1055.1%</t>
         </is>
       </c>
     </row>
@@ -2672,26 +2672,26 @@
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>490</v>
+        <v>481</v>
       </c>
       <c r="F15" s="9" t="n">
-        <v>930</v>
+        <v>912</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>1531</v>
+        <v>1501</v>
       </c>
       <c r="H15" s="9" t="n">
-        <v>2855</v>
+        <v>2778</v>
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>1279.2%</t>
+          <t>1268.5%</t>
         </is>
       </c>
     </row>
@@ -2707,26 +2707,26 @@
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>862</v>
+        <v>811</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>1302</v>
+        <v>1232</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>2304</v>
+        <v>2202</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>4521</v>
+        <v>4326</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>10810</v>
+        <v>10506</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>28569</v>
+        <v>27891</v>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>3214.3%</t>
+          <t>3339.1%</t>
         </is>
       </c>
     </row>
@@ -2742,26 +2742,26 @@
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>1513</v>
+        <v>1453</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>2094</v>
+        <v>1989</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>3108</v>
+        <v>2883</v>
       </c>
       <c r="F17" s="9" t="n">
-        <v>5520</v>
+        <v>5157</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>10682</v>
+        <v>10088</v>
       </c>
       <c r="H17" s="9" t="n">
-        <v>25379</v>
+        <v>24208</v>
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>1577.4%</t>
+          <t>1566.1%</t>
         </is>
       </c>
     </row>
@@ -2777,26 +2777,26 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>800</v>
+        <v>681</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>974</v>
+        <v>814</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>1274</v>
+        <v>1054</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>1510</v>
+        <v>1264</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>1758</v>
+        <v>1494</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>1946</v>
+        <v>1663</v>
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>143.2%</t>
+          <t>144.2%</t>
         </is>
       </c>
     </row>
@@ -2812,26 +2812,26 @@
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>710</v>
+        <v>628</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>1191</v>
+        <v>1075</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>2195</v>
+        <v>1982</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>3517</v>
+        <v>3157</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>6524</v>
+        <v>5955</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>15520</v>
+        <v>14583</v>
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>2085.9%</t>
+          <t>2222.1%</t>
         </is>
       </c>
     </row>
@@ -2847,26 +2847,26 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>756</v>
+        <v>624</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>1091</v>
+        <v>926</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>1853</v>
+        <v>1612</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>3206</v>
+        <v>2823</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>5711</v>
+        <v>5088</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>12811</v>
+        <v>11651</v>
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>1594.6%</t>
+          <t>1767.1%</t>
         </is>
       </c>
     </row>
@@ -2882,26 +2882,26 @@
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>407</v>
+        <v>386</v>
       </c>
       <c r="D21" s="9" t="n">
-        <v>538</v>
+        <v>513</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>758</v>
+        <v>725</v>
       </c>
       <c r="F21" s="9" t="n">
-        <v>1291</v>
+        <v>1246</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>2490</v>
+        <v>2425</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>5668</v>
+        <v>5512</v>
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>1292.6%</t>
+          <t>1328.0%</t>
         </is>
       </c>
     </row>
@@ -2917,26 +2917,26 @@
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>6067</v>
+        <v>5319</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>9122</v>
+        <v>8166</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>12974</v>
+        <v>11782</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>19678</v>
+        <v>18205</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>28926</v>
+        <v>27203</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>48784</v>
+        <v>46738</v>
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>704.1%</t>
+          <t>778.7%</t>
         </is>
       </c>
     </row>
@@ -3018,26 +3018,26 @@
       </c>
       <c r="B25" s="9" t="n"/>
       <c r="C25" s="9" t="n">
-        <v>23189</v>
+        <v>19426</v>
       </c>
       <c r="D25" s="9" t="n">
-        <v>34958</v>
+        <v>29807</v>
       </c>
       <c r="E25" s="9" t="n">
-        <v>56576</v>
+        <v>49263</v>
       </c>
       <c r="F25" s="9" t="n">
-        <v>106127</v>
+        <v>95255</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>206297</v>
+        <v>189865</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>464866</v>
+        <v>434327</v>
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>1904.7%</t>
+          <t>2135.8%</t>
         </is>
       </c>
     </row>

</xml_diff>